<commit_message>
Cambios en datasets, y eliminacion de outputs
</commit_message>
<xml_diff>
--- a/data/Raw/ventas_enero.xlsx
+++ b/data/Raw/ventas_enero.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\power\OneDrive\Escritorio\archivos_t\Proyectos\Proyecto Informe ventas\data\Raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06266B45-184A-434C-9B0C-BA972197445F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28A2AA83-26E5-4A0D-BD14-80F9EC823F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
   <si>
     <t>Fecha</t>
   </si>
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -482,74 +482,222 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
-        <v>45667</v>
+        <v>45681</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="1">
+        <v>150000</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
-        <v>45681</v>
+        <v>45686</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" s="1">
-        <v>150000</v>
+        <v>2750000</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
-        <v>45686</v>
+        <v>45677</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="1">
-        <v>2750000</v>
+        <v>20000</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
-        <v>45677</v>
+        <v>45669</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D8" s="1">
-        <v>20000</v>
+        <v>74000</v>
       </c>
       <c r="E8">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
+        <v>45686</v>
+      </c>
+      <c r="B9">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="1">
+        <v>2750000</v>
+      </c>
+      <c r="E9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>45677</v>
+      </c>
+      <c r="B10">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="1">
+        <v>20000</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>45686</v>
+      </c>
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2750000</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>45677</v>
+      </c>
+      <c r="B12">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="1">
+        <v>20000</v>
+      </c>
+      <c r="E12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
         <v>45669</v>
       </c>
-      <c r="B9">
+      <c r="B13">
         <v>3</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C13" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D13" s="1">
         <v>74000</v>
       </c>
-      <c r="E9">
+      <c r="E13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>45669</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1">
+        <v>74000</v>
+      </c>
+      <c r="E14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>45686</v>
+      </c>
+      <c r="B15">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2750000</v>
+      </c>
+      <c r="E15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>45677</v>
+      </c>
+      <c r="B16">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="1">
+        <v>20000</v>
+      </c>
+      <c r="E16">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>45669</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="1">
+        <v>74000</v>
+      </c>
+      <c r="E17">
         <v>8</v>
       </c>
     </row>

</xml_diff>